<commit_message>
Restore tables and figures from pre-placeholder state
- Restore 44 .tex tables from commit e72488de (before placeholder conversion)
- Restore 25 PNG figures including RQ1a enhanced_analysis_latest images
- Regenerate sensitivity analysis with proper prompt distances
- All thesis assets now compile correctly (272 pages)
</commit_message>
<xml_diff>
--- a/final_runs/RQ1b_corrector_ablation/corrector_ablation_groundtruth_results.xlsx
+++ b/final_runs/RQ1b_corrector_ablation/corrector_ablation_groundtruth_results.xlsx
@@ -5527,107 +5527,107 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>F1_Delta_min</t>
+          <t>F1_Delta_count</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>F1_Delta_max</t>
+          <t>Precision_Delta</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Precision_Delta</t>
+          <t>Precision_Delta_std</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Precision_Delta_std</t>
+          <t>Precision_Delta_count</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Precision_Delta_min</t>
+          <t>Recall_Delta</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Precision_Delta_max</t>
+          <t>Recall_Delta_std</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Recall_Delta</t>
+          <t>Recall_Delta_count</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Recall_Delta_std</t>
+          <t>Judge_Score_Delta</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Recall_Delta_min</t>
+          <t>Judge_Score_Delta_std</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Recall_Delta_max</t>
+          <t>Judge_Score_Delta_count</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Judge_Score_Delta</t>
+          <t>Actions_Total_sum</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Judge_Score_Delta_std</t>
+          <t>Actions_Revise_sum</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Judge_Score_Delta_min</t>
+          <t>Actions_Change_sum</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Judge_Score_Delta_max</t>
+          <t>Actions_None_sum</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Actions_Total_sum</t>
+          <t>Actions_Error_sum</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Actions_Revise_sum</t>
+          <t>Actions_Remove_sum</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Actions_Change_sum</t>
+          <t>Actions_Flip_sum</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Actions_None_sum</t>
+          <t>F1_Delta_ci</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Actions_Error_sum</t>
+          <t>Precision_Delta_ci</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Actions_Remove_sum</t>
+          <t>Recall_Delta_ci</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>Actions_Flip_sum</t>
+          <t>Judge_Score_Delta_ci</t>
         </is>
       </c>
     </row>
@@ -5649,67 +5649,67 @@
         <v>0.004570557952810574</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.0406</v>
+        <v>3</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.0315</v>
+        <v>-0.04323333333333334</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.04323333333333334</v>
+        <v>0.004219399641339196</v>
       </c>
       <c r="H2" t="n">
-        <v>0.004219399641339196</v>
+        <v>3</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.0472</v>
+        <v>0.0294</v>
       </c>
       <c r="J2" t="n">
-        <v>-0.0388</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0294</v>
+        <v>3</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>0.09999999999999994</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0294</v>
+        <v>0.004761904761904785</v>
       </c>
       <c r="N2" t="n">
-        <v>0.0294</v>
+        <v>3</v>
       </c>
       <c r="O2" t="n">
-        <v>0.09999999999999994</v>
+        <v>81</v>
       </c>
       <c r="P2" t="n">
-        <v>0.004761904761904785</v>
+        <v>44</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.09523809523809512</v>
+        <v>37</v>
       </c>
       <c r="R2" t="n">
-        <v>0.1047619047619047</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>0</v>
+        <v>0.01135389537417643</v>
       </c>
       <c r="W2" t="n">
-        <v>0</v>
+        <v>0.01048156976986662</v>
       </c>
       <c r="X2" t="n">
         <v>0</v>
       </c>
       <c r="Y2" t="n">
-        <v>0</v>
+        <v>0.01182922719866456</v>
       </c>
     </row>
     <row r="3">
@@ -5730,67 +5730,67 @@
         <v>0.006954135460285482</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0239</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0377</v>
+        <v>0.0097</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0097</v>
+        <v>0.003555277766926236</v>
       </c>
       <c r="H3" t="n">
-        <v>0.003555277766926236</v>
+        <v>3</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0069</v>
+        <v>0.1313333333333333</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0137</v>
+        <v>0.02312019319411785</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1313333333333333</v>
+        <v>3</v>
       </c>
       <c r="L3" t="n">
-        <v>0.02312019319411785</v>
+        <v>0.07873315852833958</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1061</v>
+        <v>0.004362985159763979</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1515</v>
+        <v>3</v>
       </c>
       <c r="O3" t="n">
-        <v>0.07873315852833958</v>
+        <v>301</v>
       </c>
       <c r="P3" t="n">
-        <v>0.004362985159763979</v>
+        <v>71</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.07521008403361285</v>
+        <v>228</v>
       </c>
       <c r="R3" t="n">
-        <v>0.08361344537815185</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>301</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>228</v>
+        <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>0</v>
+        <v>0.01727503014930133</v>
       </c>
       <c r="W3" t="n">
-        <v>0</v>
+        <v>0.008831799576459515</v>
       </c>
       <c r="X3" t="n">
-        <v>0</v>
+        <v>0.05743374381574972</v>
       </c>
       <c r="Y3" t="n">
-        <v>0</v>
+        <v>0.01083825597104243</v>
       </c>
     </row>
     <row r="4">
@@ -5811,67 +5811,67 @@
         <v>0.07669461084935064</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.1271</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0242</v>
+        <v>-0.1136666666666667</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.1136666666666667</v>
+        <v>0.06963334928992956</v>
       </c>
       <c r="H4" t="n">
-        <v>0.06963334928992956</v>
+        <v>3</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.1888</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="J4" t="n">
-        <v>-0.0513</v>
+        <v>0.08335000499900004</v>
       </c>
       <c r="K4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L4" t="n">
         <v>0.08333333333333333</v>
       </c>
-      <c r="L4" t="n">
-        <v>0.08335000499900004</v>
-      </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>0.02099455524325894</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1667</v>
+        <v>3</v>
       </c>
       <c r="O4" t="n">
-        <v>0.08333333333333333</v>
+        <v>36</v>
       </c>
       <c r="P4" t="n">
-        <v>0.02099455524325894</v>
+        <v>7</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0590909090909093</v>
+        <v>26</v>
       </c>
       <c r="R4" t="n">
-        <v>0.09545454545454546</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>0</v>
+        <v>0.190519975096527</v>
       </c>
       <c r="W4" t="n">
-        <v>0</v>
+        <v>0.1729788289644535</v>
       </c>
       <c r="X4" t="n">
-        <v>0</v>
+        <v>0.2070528906900287</v>
       </c>
       <c r="Y4" t="n">
-        <v>0</v>
+        <v>0.05215336642055884</v>
       </c>
     </row>
     <row r="5">
@@ -5892,53 +5892,57 @@
         <v>0.003758102358017051</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.0283</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.021</v>
+        <v>-0.0311</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.0311</v>
+        <v>0.003764306044943744</v>
       </c>
       <c r="H5" t="n">
-        <v>0.003764306044943744</v>
+        <v>3</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.0352</v>
+        <v>0.0294</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.0278</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0294</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.0294</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>0.0294</v>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>80</v>
+      </c>
+      <c r="P5" t="n">
+        <v>52</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>28</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
       <c r="S5" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="U5" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="V5" t="n">
-        <v>0</v>
+        <v>0.009335643792052307</v>
       </c>
       <c r="W5" t="n">
-        <v>0</v>
+        <v>0.009351054604698605</v>
       </c>
       <c r="X5" t="n">
         <v>0</v>
@@ -5965,56 +5969,60 @@
         <v>0.003807011076071796</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0217</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0293</v>
+        <v>0.007233333333333334</v>
       </c>
       <c r="G6" t="n">
-        <v>0.007233333333333334</v>
+        <v>0.003257811126098831</v>
       </c>
       <c r="H6" t="n">
-        <v>0.003257811126098831</v>
+        <v>3</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0035</v>
+        <v>0.1161666666666667</v>
       </c>
       <c r="J6" t="n">
-        <v>0.0095</v>
+        <v>0.00871798906476335</v>
       </c>
       <c r="K6" t="n">
-        <v>0.1161666666666667</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.00871798906476335</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0.1061</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
-        <v>0.1212</v>
-      </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>292</v>
+      </c>
+      <c r="P6" t="n">
+        <v>78</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>214</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
       <c r="S6" t="n">
-        <v>292</v>
+        <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="U6" t="n">
-        <v>214</v>
+        <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>0</v>
+        <v>0.009457139783003957</v>
       </c>
       <c r="W6" t="n">
-        <v>0</v>
+        <v>0.008092851476001627</v>
       </c>
       <c r="X6" t="n">
-        <v>0</v>
+        <v>0.02165668540613725</v>
       </c>
       <c r="Y6" t="n">
         <v>0</v>
@@ -6038,62 +6046,62 @@
         <v>0.06813156390396451</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.105</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0242</v>
+        <v>-0.09216666666666667</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.09216666666666667</v>
+        <v>0.0603636756115243</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0603636756115243</v>
+        <v>3</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.1615</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.0513</v>
+        <v>0.08335000499900004</v>
       </c>
       <c r="K7" t="n">
-        <v>0.08333333333333333</v>
+        <v>3</v>
       </c>
       <c r="L7" t="n">
-        <v>0.08335000499900004</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
+        <v>0.06809841534612182</v>
+      </c>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>0.1667</v>
+        <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>0.06809841534612182</v>
-      </c>
-      <c r="P7" t="inlineStr"/>
+        <v>36</v>
+      </c>
+      <c r="P7" t="n">
+        <v>14</v>
+      </c>
       <c r="Q7" t="n">
-        <v>0.06809841534612182</v>
+        <v>22</v>
       </c>
       <c r="R7" t="n">
-        <v>0.06809841534612182</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>0</v>
+        <v>0.1692481872522684</v>
       </c>
       <c r="W7" t="n">
-        <v>0</v>
+        <v>0.1499516830045929</v>
       </c>
       <c r="X7" t="n">
-        <v>0</v>
+        <v>0.2070528906900287</v>
       </c>
       <c r="Y7" t="n">
         <v>0</v>
@@ -6117,67 +6125,67 @@
         <v>0.002413158373031768</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.049</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.0443</v>
+        <v>-0.0537</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.0537</v>
+        <v>0.002551470164434614</v>
       </c>
       <c r="H8" t="n">
-        <v>0.002551470164434614</v>
+        <v>3</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.0556</v>
+        <v>0.0294</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.0508</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0294</v>
+        <v>3</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>0.1007936507936508</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0294</v>
+        <v>0.004956347617776595</v>
       </c>
       <c r="N8" t="n">
-        <v>0.0294</v>
+        <v>3</v>
       </c>
       <c r="O8" t="n">
-        <v>0.1007936507936508</v>
+        <v>81</v>
       </c>
       <c r="P8" t="n">
-        <v>0.004956347617776595</v>
+        <v>34</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.09523809523809512</v>
+        <v>46</v>
       </c>
       <c r="R8" t="n">
-        <v>0.1047619047619047</v>
+        <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="U8" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>0</v>
+        <v>0.005994617718799998</v>
       </c>
       <c r="W8" t="n">
-        <v>0</v>
+        <v>0.006338203255799297</v>
       </c>
       <c r="X8" t="n">
         <v>0</v>
       </c>
       <c r="Y8" t="n">
-        <v>0</v>
+        <v>0.01231225002971017</v>
       </c>
     </row>
     <row r="9">
@@ -6198,67 +6206,67 @@
         <v>0.00357957166897568</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0196</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0258</v>
+        <v>0.0046</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0046</v>
+        <v>0.00272213151776324</v>
       </c>
       <c r="H9" t="n">
-        <v>0.00272213151776324</v>
+        <v>3</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0017</v>
+        <v>0.1262666666666667</v>
       </c>
       <c r="J9" t="n">
-        <v>0.0071</v>
+        <v>0.008775724091682306</v>
       </c>
       <c r="K9" t="n">
-        <v>0.1262666666666667</v>
+        <v>3</v>
       </c>
       <c r="L9" t="n">
-        <v>0.008775724091682306</v>
+        <v>0.07649120084186589</v>
       </c>
       <c r="M9" t="n">
-        <v>0.1212</v>
+        <v>0.002750738839711521</v>
       </c>
       <c r="N9" t="n">
-        <v>0.1364</v>
+        <v>3</v>
       </c>
       <c r="O9" t="n">
-        <v>0.07649120084186589</v>
+        <v>301</v>
       </c>
       <c r="P9" t="n">
-        <v>0.002750738839711521</v>
+        <v>38</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.07394957983193207</v>
+        <v>255</v>
       </c>
       <c r="R9" t="n">
-        <v>0.07941176470588218</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>301</v>
+        <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>255</v>
+        <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>0</v>
+        <v>0.008892148974705361</v>
       </c>
       <c r="W9" t="n">
-        <v>0</v>
+        <v>0.006762149559536029</v>
       </c>
       <c r="X9" t="n">
-        <v>0</v>
+        <v>0.02180010716379377</v>
       </c>
       <c r="Y9" t="n">
-        <v>0</v>
+        <v>0.006833214086819056</v>
       </c>
     </row>
     <row r="10">
@@ -6279,67 +6287,67 @@
         <v>0.06545464078275887</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1271</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>-0.0959</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.0959</v>
+        <v>0.09443574535100573</v>
       </c>
       <c r="H10" t="n">
-        <v>0.09443574535100573</v>
+        <v>3</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.1888</v>
+        <v>0.02776666666666667</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>0.04809327742349583</v>
       </c>
       <c r="K10" t="n">
-        <v>0.02776666666666667</v>
+        <v>3</v>
       </c>
       <c r="L10" t="n">
-        <v>0.04809327742349583</v>
+        <v>0.09242424242424241</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>0.02148098011932997</v>
       </c>
       <c r="N10" t="n">
-        <v>0.0833</v>
+        <v>3</v>
       </c>
       <c r="O10" t="n">
-        <v>0.09242424242424241</v>
+        <v>36</v>
       </c>
       <c r="P10" t="n">
-        <v>0.02148098011932997</v>
+        <v>8</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.06818181818181823</v>
+        <v>28</v>
       </c>
       <c r="R10" t="n">
-        <v>0.109090909090909</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>0</v>
+        <v>0.1625983415755075</v>
       </c>
       <c r="W10" t="n">
-        <v>0</v>
+        <v>0.2345913963607771</v>
       </c>
       <c r="X10" t="n">
-        <v>0</v>
+        <v>0.1194703241278962</v>
       </c>
       <c r="Y10" t="n">
-        <v>0</v>
+        <v>0.0533617127991254</v>
       </c>
     </row>
   </sheetData>
@@ -6374,107 +6382,107 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>F1_Delta_min</t>
+          <t>F1_Delta_count</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>F1_Delta_max</t>
+          <t>Precision_Delta_mean</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Precision_Delta_mean</t>
+          <t>Precision_Delta_std</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Precision_Delta_std</t>
+          <t>Precision_Delta_count</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Precision_Delta_min</t>
+          <t>Recall_Delta_mean</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Precision_Delta_max</t>
+          <t>Recall_Delta_std</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Recall_Delta_mean</t>
+          <t>Recall_Delta_count</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Recall_Delta_std</t>
+          <t>Judge_Score_Delta_mean</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Recall_Delta_min</t>
+          <t>Judge_Score_Delta_std</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Recall_Delta_max</t>
+          <t>Judge_Score_Delta_count</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Judge_Score_Delta_mean</t>
+          <t>Actions_Total_sum_sum</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Judge_Score_Delta_std</t>
+          <t>Actions_Revise_sum_sum</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Judge_Score_Delta_min</t>
+          <t>Actions_Change_sum_sum</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Judge_Score_Delta_max</t>
+          <t>Actions_None_sum_sum</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Actions_Total_sum_sum</t>
+          <t>Actions_Error_sum_sum</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Actions_Revise_sum_sum</t>
+          <t>Actions_Remove_sum_sum</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Actions_Change_sum_sum</t>
+          <t>Actions_Flip_sum_sum</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Actions_None_sum_sum</t>
+          <t>F1_Delta_ci</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Actions_Error_sum_sum</t>
+          <t>Precision_Delta_ci</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Actions_Remove_sum_sum</t>
+          <t>Recall_Delta_ci</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Actions_Flip_sum_sum</t>
+          <t>Judge_Score_Delta_ci</t>
         </is>
       </c>
     </row>
@@ -6491,67 +6499,67 @@
         <v>0.04091195605380105</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.04416666666666667</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0303</v>
+        <v>-0.04906666666666667</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.04906666666666667</v>
+        <v>0.06188985736325819</v>
       </c>
       <c r="G2" t="n">
-        <v>0.06188985736325819</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.1136666666666667</v>
+        <v>0.08135555555555556</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0097</v>
+        <v>0.05099543915699535</v>
       </c>
       <c r="J2" t="n">
-        <v>0.08135555555555556</v>
+        <v>3</v>
       </c>
       <c r="K2" t="n">
-        <v>0.05099543915699535</v>
+        <v>0.08735549728722429</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0294</v>
+        <v>0.01118941413565375</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1313333333333333</v>
+        <v>3</v>
       </c>
       <c r="N2" t="n">
-        <v>0.08735549728722429</v>
+        <v>418</v>
       </c>
       <c r="O2" t="n">
-        <v>0.01118941413565375</v>
+        <v>122</v>
       </c>
       <c r="P2" t="n">
-        <v>0.07873315852833958</v>
+        <v>291</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.09999999999999994</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>418</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>122</v>
+        <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>291</v>
+        <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>0</v>
+        <v>0.1016309328934599</v>
       </c>
       <c r="V2" t="n">
-        <v>0</v>
+        <v>0.1537429286490133</v>
       </c>
       <c r="W2" t="n">
-        <v>0</v>
+        <v>0.1266796935355917</v>
       </c>
       <c r="X2" t="n">
-        <v>0</v>
+        <v>0.02779604562642525</v>
       </c>
     </row>
     <row r="3">
@@ -6567,62 +6575,62 @@
         <v>0.02987955451103275</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0279</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02563333333333333</v>
+        <v>-0.03867777777777778</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.03867777777777778</v>
+        <v>0.05013139771677065</v>
       </c>
       <c r="G3" t="n">
-        <v>0.05013139771677065</v>
+        <v>3</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.09216666666666667</v>
+        <v>0.07629999999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>0.007233333333333334</v>
+        <v>0.04380883979797279</v>
       </c>
       <c r="J3" t="n">
-        <v>0.07629999999999999</v>
+        <v>3</v>
       </c>
       <c r="K3" t="n">
-        <v>0.04380883979797279</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.0294</v>
-      </c>
+        <v>0.06809841534612182</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
-        <v>0.1161666666666667</v>
+        <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>0.06809841534612182</v>
-      </c>
-      <c r="O3" t="inlineStr"/>
+        <v>408</v>
+      </c>
+      <c r="O3" t="n">
+        <v>144</v>
+      </c>
       <c r="P3" t="n">
-        <v>0.06809841534612182</v>
+        <v>264</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.06809841534612182</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>408</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>144</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>264</v>
+        <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0</v>
+        <v>0.07422492817023633</v>
       </c>
       <c r="V3" t="n">
-        <v>0</v>
+        <v>0.1245332956094411</v>
       </c>
       <c r="W3" t="n">
-        <v>0</v>
+        <v>0.1088271910488243</v>
       </c>
       <c r="X3" t="n">
         <v>0</v>
@@ -6641,67 +6649,67 @@
         <v>0.04315803431489814</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.05449999999999999</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>0.02373333333333333</v>
+        <v>-0.04833333333333333</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.04833333333333333</v>
+        <v>0.05046447595421291</v>
       </c>
       <c r="G4" t="n">
-        <v>0.05046447595421291</v>
+        <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.0959</v>
+        <v>0.06114444444444445</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0046</v>
+        <v>0.05640341137568556</v>
       </c>
       <c r="J4" t="n">
-        <v>0.06114444444444445</v>
+        <v>3</v>
       </c>
       <c r="K4" t="n">
-        <v>0.05640341137568556</v>
+        <v>0.08990303135325305</v>
       </c>
       <c r="L4" t="n">
-        <v>0.02776666666666667</v>
+        <v>0.01234583522339062</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1262666666666667</v>
+        <v>3</v>
       </c>
       <c r="N4" t="n">
-        <v>0.08990303135325305</v>
+        <v>418</v>
       </c>
       <c r="O4" t="n">
-        <v>0.01234583522339062</v>
+        <v>80</v>
       </c>
       <c r="P4" t="n">
-        <v>0.07649120084186589</v>
+        <v>329</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.1007936507936508</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>418</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>329</v>
+        <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>0</v>
+        <v>0.1072105006053247</v>
       </c>
       <c r="V4" t="n">
-        <v>0</v>
+        <v>0.1253607078200245</v>
       </c>
       <c r="W4" t="n">
-        <v>0</v>
+        <v>0.1401138412679717</v>
       </c>
       <c r="X4" t="n">
-        <v>0</v>
+        <v>0.03066875486110014</v>
       </c>
     </row>
   </sheetData>

</xml_diff>